<commit_message>
Update ingevulde beoordeling Leon.xlsx
</commit_message>
<xml_diff>
--- a/bestanden/ingevulde beoordeling Leon.xlsx
+++ b/bestanden/ingevulde beoordeling Leon.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonb\OneDrive\Documenten\GitHub\The-Hollow-Throne\bestanden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE5A29-6E31-4BF5-89B5-E8ADB9D93043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9F8F16-7175-49C5-B60A-D80E07AE421C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1006,35 +1006,35 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1412,10 +1412,10 @@
       <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="40"/>
+      <c r="D2" s="48"/>
       <c r="E2" s="24" t="s">
         <v>2</v>
       </c>
@@ -1449,7 +1449,7 @@
       </c>
     </row>
     <row r="4" spans="2:8" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="39" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="27" t="s">
@@ -1464,14 +1464,14 @@
       <c r="F4" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="43">
+      <c r="G4" s="41">
         <f>IF(C5=TRUE,0,IF(D5=TRUE,1,IF(E5=TRUE,2,IF(F5=TRUE,3,"leeg"))))</f>
         <v>3</v>
       </c>
-      <c r="H4" s="44"/>
+      <c r="H4" s="42"/>
     </row>
     <row r="5" spans="2:8" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="42"/>
+      <c r="B5" s="40"/>
       <c r="C5" s="30" t="b">
         <v>0</v>
       </c>
@@ -1484,11 +1484,11 @@
       <c r="F5" s="32" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="2:8" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="43" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="10" t="s">
@@ -1503,14 +1503,14 @@
       <c r="F6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="47">
+      <c r="G6" s="45">
         <f t="shared" ref="G6" si="0">IF(C7=TRUE,0,IF(D7=TRUE,1,IF(E7=TRUE,2,IF(F7=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H6" s="48"/>
+      <c r="H6" s="46"/>
     </row>
     <row r="7" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="46"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="12" t="b">
         <v>0</v>
       </c>
@@ -1523,11 +1523,11 @@
       <c r="F7" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="46"/>
     </row>
     <row r="8" spans="2:8" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="39" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="27" t="s">
@@ -1542,14 +1542,14 @@
       <c r="F8" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="41">
         <f t="shared" ref="G8" si="1">IF(C9=TRUE,0,IF(D9=TRUE,1,IF(E9=TRUE,2,IF(F9=TRUE,3,"leeg"))))</f>
         <v>3</v>
       </c>
-      <c r="H8" s="44"/>
+      <c r="H8" s="42"/>
     </row>
     <row r="9" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="42"/>
+      <c r="B9" s="40"/>
       <c r="C9" s="30" t="b">
         <v>0</v>
       </c>
@@ -1562,11 +1562,11 @@
       <c r="F9" s="34" t="b">
         <v>1</v>
       </c>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="42"/>
     </row>
     <row r="10" spans="2:8" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="43" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="10" t="s">
@@ -1581,14 +1581,14 @@
       <c r="F10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="47">
+      <c r="G10" s="45">
         <f t="shared" ref="G10" si="2">IF(C11=TRUE,0,IF(D11=TRUE,1,IF(E11=TRUE,2,IF(F11=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H10" s="48"/>
+      <c r="H10" s="46"/>
     </row>
     <row r="11" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
+      <c r="B11" s="44"/>
       <c r="C11" s="12" t="b">
         <v>0</v>
       </c>
@@ -1601,11 +1601,11 @@
       <c r="F11" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="G11" s="47"/>
-      <c r="H11" s="48"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="46"/>
     </row>
     <row r="12" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="39" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="27" t="s">
@@ -1620,14 +1620,14 @@
       <c r="F12" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="43">
+      <c r="G12" s="41">
         <f t="shared" ref="G12" si="3">IF(C13=TRUE,0,IF(D13=TRUE,1,IF(E13=TRUE,2,IF(F13=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H12" s="44"/>
+      <c r="H12" s="42"/>
     </row>
     <row r="13" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="42"/>
+      <c r="B13" s="40"/>
       <c r="C13" s="30" t="b">
         <v>0</v>
       </c>
@@ -1640,11 +1640,11 @@
       <c r="F13" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="42"/>
     </row>
     <row r="14" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="45" t="s">
+      <c r="B14" s="43" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="10" t="s">
@@ -1659,14 +1659,14 @@
       <c r="F14" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="G14" s="47">
+      <c r="G14" s="45">
         <f t="shared" ref="G14" si="4">IF(C15=TRUE,0,IF(D15=TRUE,1,IF(E15=TRUE,2,IF(F15=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H14" s="48"/>
+      <c r="H14" s="46"/>
     </row>
     <row r="15" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="46"/>
+      <c r="B15" s="44"/>
       <c r="C15" s="12" t="b">
         <v>0</v>
       </c>
@@ -1679,11 +1679,11 @@
       <c r="F15" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="G15" s="47"/>
-      <c r="H15" s="48"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
     </row>
     <row r="16" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="39" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="27" t="s">
@@ -1698,14 +1698,14 @@
       <c r="F16" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="43">
+      <c r="G16" s="41">
         <f t="shared" ref="G16" si="5">IF(C17=TRUE,0,IF(D17=TRUE,1,IF(E17=TRUE,2,IF(F17=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H16" s="44"/>
+      <c r="H16" s="42"/>
     </row>
     <row r="17" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="42"/>
+      <c r="B17" s="40"/>
       <c r="C17" s="30" t="b">
         <v>0</v>
       </c>
@@ -1718,11 +1718,11 @@
       <c r="F17" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="42"/>
     </row>
     <row r="18" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="45" t="s">
+      <c r="B18" s="43" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="10" t="s">
@@ -1737,14 +1737,14 @@
       <c r="F18" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="47">
+      <c r="G18" s="45">
         <f t="shared" ref="G18" si="6">IF(C19=TRUE,0,IF(D19=TRUE,1,IF(E19=TRUE,2,IF(F19=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H18" s="48"/>
+      <c r="H18" s="46"/>
     </row>
     <row r="19" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="46"/>
+      <c r="B19" s="44"/>
       <c r="C19" s="12" t="b">
         <v>0</v>
       </c>
@@ -1757,11 +1757,11 @@
       <c r="F19" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="46"/>
     </row>
     <row r="20" spans="2:8" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="39" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="27" t="s">
@@ -1776,14 +1776,14 @@
       <c r="F20" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="43">
+      <c r="G20" s="41">
         <f t="shared" ref="G20" si="7">IF(C21=TRUE,0,IF(D21=TRUE,1,IF(E21=TRUE,2,IF(F21=TRUE,3,"leeg"))))</f>
         <v>2</v>
       </c>
-      <c r="H20" s="44"/>
+      <c r="H20" s="42"/>
     </row>
     <row r="21" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="42"/>
+      <c r="B21" s="40"/>
       <c r="C21" s="30" t="b">
         <v>0</v>
       </c>
@@ -1796,11 +1796,11 @@
       <c r="F21" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="G21" s="43"/>
-      <c r="H21" s="44"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="42"/>
     </row>
     <row r="22" spans="2:8" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="B22" s="45" t="s">
+      <c r="B22" s="43" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="10" t="s">
@@ -1815,33 +1815,33 @@
       <c r="F22" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G22" s="47">
+      <c r="G22" s="45">
         <f t="shared" ref="G22" si="8">IF(C23=TRUE,0,IF(D23=TRUE,1,IF(E23=TRUE,2,IF(F23=TRUE,3,"leeg"))))</f>
+        <v>2</v>
+      </c>
+      <c r="H22" s="46" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="44"/>
+      <c r="C23" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="13" t="b">
         <v>1</v>
       </c>
-      <c r="H22" s="48" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="46"/>
-      <c r="C23" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D23" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E23" s="13" t="b">
-        <v>0</v>
-      </c>
       <c r="F23" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="G23" s="47"/>
-      <c r="H23" s="48"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="46"/>
     </row>
     <row r="24" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="39" t="s">
         <v>46</v>
       </c>
       <c r="C24" s="27" t="s">
@@ -1856,14 +1856,14 @@
       <c r="F24" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="G24" s="43">
+      <c r="G24" s="41">
         <f t="shared" ref="G24" si="9">IF(C25=TRUE,0,IF(D25=TRUE,1,IF(E25=TRUE,2,IF(F25=TRUE,3,"leeg"))))</f>
         <v>3</v>
       </c>
-      <c r="H24" s="44"/>
+      <c r="H24" s="42"/>
     </row>
     <row r="25" spans="2:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="42"/>
+      <c r="B25" s="40"/>
       <c r="C25" s="30" t="b">
         <v>0</v>
       </c>
@@ -1876,8 +1876,8 @@
       <c r="F25" s="32" t="b">
         <v>1</v>
       </c>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="42"/>
     </row>
     <row r="26" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="18"/>
@@ -1889,12 +1889,37 @@
       </c>
       <c r="G26" s="22" t="str">
         <f>IF(COUNTIFS(G4:G25,"leeg")&gt;0," ",IF(COUNTIFS(G4:G25,0)&gt;0,"O",IF(COUNTIFS(G4:G25,1)&gt;0,"O",IF(COUNTIFS(G4:G25,3)&gt;7,"G","V"))))</f>
-        <v>O</v>
+        <v>V</v>
       </c>
       <c r="H26" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="G24:G25"/>
     <mergeCell ref="H24:H25"/>
@@ -1904,31 +1929,6 @@
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="H22:H23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="G12:G13"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
   </mergeCells>
   <conditionalFormatting sqref="G26">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
@@ -1946,12 +1946,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fedf7ced-9c7a-48f8-a07c-98a598b105da">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="008856c5-5e82-4bb2-b94b-d933afeebe23" xsi:nil="true"/>
+    <ReferenceId xmlns="fedf7ced-9c7a-48f8-a07c-98a598b105da" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2150,21 +2153,23 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fedf7ced-9c7a-48f8-a07c-98a598b105da">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="008856c5-5e82-4bb2-b94b-d933afeebe23" xsi:nil="true"/>
-    <ReferenceId xmlns="fedf7ced-9c7a-48f8-a07c-98a598b105da" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22955E41-5EBA-4849-A6EC-932D8CFA156C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AD17981-A18F-4D0D-81EF-1093232EB82C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="094ecc41-7a37-40c9-8390-f18431712098"/>
+    <ds:schemaRef ds:uri="32dd6115-ce5d-46b4-b638-9e7d5ca6cbee"/>
+    <ds:schemaRef ds:uri="fedf7ced-9c7a-48f8-a07c-98a598b105da"/>
+    <ds:schemaRef ds:uri="008856c5-5e82-4bb2-b94b-d933afeebe23"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2189,14 +2194,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AD17981-A18F-4D0D-81EF-1093232EB82C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22955E41-5EBA-4849-A6EC-932D8CFA156C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="094ecc41-7a37-40c9-8390-f18431712098"/>
-    <ds:schemaRef ds:uri="32dd6115-ce5d-46b4-b638-9e7d5ca6cbee"/>
-    <ds:schemaRef ds:uri="fedf7ced-9c7a-48f8-a07c-98a598b105da"/>
-    <ds:schemaRef ds:uri="008856c5-5e82-4bb2-b94b-d933afeebe23"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>